<commit_message>
Review: correct #59 date; changelog
</commit_message>
<xml_diff>
--- a/napor/NAPOR_iran_war.xlsx
+++ b/napor/NAPOR_iran_war.xlsx
@@ -1140,7 +1140,7 @@
     <t xml:space="preserve">NPR 2026-07-08</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmed (NPR, Jul 8).</t>
+    <t xml:space="preserve">Confirmed (NPR, published Jul 8): NPR dates Trump's remark to Tuesday, Jul 7, so the row date was moved from Jul 8 to Jul 7 (mastermind review, Oct 22).</t>
   </si>
   <si>
     <t xml:space="preserve">Strike (major escalation)</t>
@@ -13486,12 +13486,12 @@
         <v>359</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="6" t="n">
         <v>59</v>
       </c>
       <c r="B60" s="7" t="n">
-        <v>46211</v>
+        <v>46210</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>51</v>
@@ -13539,13 +13539,13 @@
         <v>60</v>
       </c>
       <c r="R60" s="6" t="s">
-        <v>71</v>
+        <v>227</v>
       </c>
       <c r="S60" s="6" t="s">
         <v>358</v>
       </c>
       <c r="T60" s="6" t="s">
-        <v>175</v>
+        <v>359</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21450,7 +21450,7 @@
       </c>
       <c r="C17" s="7" t="n">
         <f aca="false">INDEX('Event Log'!$B$2:$B$182,MATCH(B17,'Event Log'!$A$2:$A$182,0))</f>
-        <v>46211</v>
+        <v>46210</v>
       </c>
       <c r="D17" s="6" t="str">
         <f aca="false">INDEX('Event Log'!$C$2:$C$182,MATCH(B17,'Event Log'!$A$2:$A$182,0))</f>
@@ -21477,7 +21477,7 @@
       </c>
       <c r="J17" s="6" t="n">
         <f aca="false">G17-C17</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" s="6" t="s">
         <v>859</v>
@@ -22455,7 +22455,7 @@
       </c>
       <c r="B39" s="14" t="n">
         <f aca="false">AVERAGE(J2:J37)</f>
-        <v>1.36111111111111</v>
+        <v>1.38888888888889</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22684,7 +22684,7 @@
       </c>
       <c r="C9" s="22" t="n">
         <f aca="false">AVERAGEIF('Action-Reaction Pairs'!$K$2:$K$37,A9,'Action-Reaction Pairs'!$J$2:$J$37)</f>
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="D9" s="23" t="n">
         <f aca="false">SUMPRODUCT(('Action-Reaction Pairs'!$K$2:$K$37=A9)*('Action-Reaction Pairs'!$J$2:$J$37&lt;=1))/COUNTIF('Action-Reaction Pairs'!$K$2:$K$37,A9)</f>
@@ -40149,7 +40149,7 @@
         <v>2549</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40166,7 +40166,7 @@
         <v>2550</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Tidy comments and docs; remove internal work-plan file
</commit_message>
<xml_diff>
--- a/napor/NAPOR_iran_war.xlsx
+++ b/napor/NAPOR_iran_war.xlsx
@@ -126,7 +126,7 @@
     <t xml:space="preserve">matcher.py (same folder) takes a new headline/snippet, checks it's Iran/US-war relevant, guesses which actor acted and which cost-category it falls in (Personnel/Casualty, Military/Property, Economic/Blockade, Political/Diplomatic), finds the closest past events by keyword overlap, and shows what historically followed them plus the base-rate stats for that category - all computed from the same data as the Factor Analysis sheet, so the two can never disagree. It's a keyword-rule matcher, not a trained model - with 86 events that's more honest than a model that would just memorize noise.</t>
   </si>
   <si>
-    <t xml:space="preserve">Compiled: 2026-10-26. Sources are cited per row; see Event Log column J. Rows 83-86 were added by a live scanner test (Sept 27-29). Rows 90-105 were added on Oct 11 from credible-outlet research covering Oct 2-11 (no US/Israeli strike on Iran and no Iranian strike on a US base was found in that window; the two Houthi rows are context from the separate Saudi-Houthi front). Rows 106-115 were added by the weekly agent on Oct 19 (Oct 12-18 news, plus catch-up rows for Oct 6 and Oct 8); again no US strike on Iranian territory and no Iranian strike on US forces was found, while attacks on shipping hit a record. Rows 87-89 were added by a live matcher test on genuinely new Oct 1 news - the matcher correctly classified the sanctions and diplomatic-statement rows; it fell back to a generic 'Military/Property' guess on the naval force-posture row since that's a troop deployment, not a strike, and the keyword rules don't have a dedicated bucket for that yet. Source audit: 2 events are still Pending credible sourcing and 4 are Not supported as logged (including #76, a confirmed duplicate of #75); treat those rows, and the Partly verified rows that rest on one side's claims, as leads, not findings.</t>
+    <t xml:space="preserve">Compiled: 2026-10-28. Sources are cited per row; see Event Log column J. Rows 83-86 were added by a live scanner test (Sept 27-29). Rows 90-105 were added on Oct 11 from credible-outlet research covering Oct 2-11 (no US/Israeli strike on Iran and no Iranian strike on a US base was found in that window; the two Houthi rows are context from the separate Saudi-Houthi front). Rows 106-115 were added by the weekly agent on Oct 19 (Oct 12-18 news, plus catch-up rows for Oct 6 and Oct 8); again no US strike on Iranian territory and no Iranian strike on US forces was found, while attacks on shipping hit a record. Rows 87-89 were added by a live matcher test on genuinely new Oct 1 news - the matcher correctly classified the sanctions and diplomatic-statement rows; it fell back to a generic 'Military/Property' guess on the naval force-posture row since that's a troop deployment, not a strike, and the keyword rules don't have a dedicated bucket for that yet. Source audit: 2 events are still Pending credible sourcing and 4 are Not supported as logged (including #76, a confirmed duplicate of #75); treat those rows, and the Partly verified rows that rest on one side's claims, as leads, not findings.</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -1140,7 +1140,7 @@
     <t xml:space="preserve">NPR 2026-07-08</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmed (NPR, published Jul 8): NPR dates Trump's remark to Tuesday, Jul 7, so the row date was moved from Jul 8 to Jul 7 (mastermind review, Oct 22).</t>
+    <t xml:space="preserve">Confirmed (NPR, published Jul 8): NPR dates Trump's remark to Tuesday, Jul 7, so the row date was moved from Jul 8 to Jul 7 (review, Oct 22).</t>
   </si>
   <si>
     <t xml:space="preserve">Strike (major escalation)</t>

</xml_diff>

<commit_message>
Options Explorer: plainer wording on all tabs (one word for categories, plain counts, no internal notes, simpler report card)
</commit_message>
<xml_diff>
--- a/napor/NAPOR_iran_war.xlsx
+++ b/napor/NAPOR_iran_war.xlsx
@@ -126,7 +126,7 @@
     <t xml:space="preserve">matcher.py (same folder) takes a new headline/snippet, checks it's Iran/US-war relevant, guesses which actor acted and which cost-category it falls in (Personnel/Casualty, Military/Property, Economic/Blockade, Political/Diplomatic), finds the closest past events by keyword overlap, and shows what historically followed them plus the base-rate stats for that category - all computed from the same data as the Factor Analysis sheet, so the two can never disagree. It's a keyword-rule matcher, not a trained model - with 86 events that's more honest than a model that would just memorize noise.</t>
   </si>
   <si>
-    <t xml:space="preserve">Compiled: 2026-10-28. Sources are cited per row; see Event Log column J. Rows 83-86 were added by a live scanner test (Sept 27-29). Rows 90-105 were added on Oct 11 from credible-outlet research covering Oct 2-11 (no US/Israeli strike on Iran and no Iranian strike on a US base was found in that window; the two Houthi rows are context from the separate Saudi-Houthi front). Rows 106-115 were added by the weekly agent on Oct 19 (Oct 12-18 news, plus catch-up rows for Oct 6 and Oct 8); again no US strike on Iranian territory and no Iranian strike on US forces was found, while attacks on shipping hit a record. Rows 87-89 were added by a live matcher test on genuinely new Oct 1 news - the matcher correctly classified the sanctions and diplomatic-statement rows; it fell back to a generic 'Military/Property' guess on the naval force-posture row since that's a troop deployment, not a strike, and the keyword rules don't have a dedicated bucket for that yet. Source audit: 2 events are still Pending credible sourcing and 4 are Not supported as logged (including #76, a confirmed duplicate of #75); treat those rows, and the Partly verified rows that rest on one side's claims, as leads, not findings.</t>
+    <t xml:space="preserve">Compiled: 2026-10-29. Sources are cited per row; see Event Log column J. Rows 83-86 were added by a live scanner test (Sept 27-29). Rows 90-105 were added on Oct 11 from credible-outlet research covering Oct 2-11 (no US/Israeli strike on Iran and no Iranian strike on a US base was found in that window; the two Houthi rows are context from the separate Saudi-Houthi front). Rows 106-115 were added by the weekly agent on Oct 19 (Oct 12-18 news, plus catch-up rows for Oct 6 and Oct 8); again no US strike on Iranian territory and no Iranian strike on US forces was found, while attacks on shipping hit a record. Rows 87-89 were added by a live matcher test on genuinely new Oct 1 news - the matcher correctly classified the sanctions and diplomatic-statement rows; it fell back to a generic 'Military/Property' guess on the naval force-posture row since that's a troop deployment, not a strike, and the keyword rules don't have a dedicated bucket for that yet. Source audit: 2 events are still Pending credible sourcing and 4 are Not supported as logged (including #76, a confirmed duplicate of #75); treat those rows, and the Partly verified rows that rest on one side's claims, as leads, not findings.</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -3366,7 +3366,7 @@
     <t xml:space="preserve">No direct casualties from the move itself.</t>
   </si>
   <si>
-    <t xml:space="preserve">Iran struck within 7 days after 3 of 15 past conciliatory US moves (timing only, not shown to be replies). Reply rate to diplomacy: not measured (not in the census).</t>
+    <t xml:space="preserve">Iran struck within 7 days after 3 of 15 past conciliatory US moves (timing only, not shown to be replies). Reply rate to diplomacy: not measured (not counted here).</t>
   </si>
   <si>
     <t xml:space="preserve">No interceptor use expected from the move itself.</t>
@@ -3588,7 +3588,7 @@
     <t xml:space="preserve">Shipping attacks have kept coming without any new US move (see the baseline line). Trump has said there will be no US strikes before Nov 3; what Iran does if that holds is not in the data.</t>
   </si>
   <si>
-    <t xml:space="preserve">Diplomatic moves are not in the census, so there is no reply rate. The last rounds (Sep 23 - Oct 9) drew rejections and counter-offers, not attacks. Iran called the US answer 'insufficient' (Oct 11) and on Oct 18 said it was still reviewing US 'comments'.</t>
+    <t xml:space="preserve">Diplomatic moves are not counted as past cases with a reply test, so there is no reply rate. The last rounds (Sep 23 - Oct 9) drew rejections and counter-offers, not attacks. Iran called the US answer 'insufficient' (Oct 11) and on Oct 18 said it was still reviewing US 'comments'.</t>
   </si>
   <si>
     <t xml:space="preserve">0 of 9 (0%)</t>
@@ -3639,7 +3639,7 @@
     <t xml:space="preserve">#33, #35, #37, #221, #264, #265 (+ unclear: #104)</t>
   </si>
   <si>
-    <t xml:space="preserve">Small sample. The pre-war cases (a 2020 fuel-cargo seizure and two seizures of Iranian arms bound for the Houthis, 2020 and 2023) drew no reply. In 2026, Iran answered the blockade start and a ship seizure, but not a warship transit. The Oct 10-11 strike on a blockade runner drew no Iranian attack on US forces within 5 days (F001: NO), but attacks on commercial shipping surged; how to score it is waiting for Sidd (census row #104 is 'Unclear').</t>
+    <t xml:space="preserve">Small sample. The pre-war cases (a 2020 fuel-cargo seizure and two seizures of Iranian arms bound for the Houthis, 2020 and 2023) drew no reply. In 2026, Iran answered the blockade start and a ship seizure, but not a warship transit. The Oct 10-11 strike on a blockade runner drew no Iranian attack on US forces within 5 days (F001: NO), but attacks on commercial shipping surged; it is not counted until the link is settled (#104).</t>
   </si>
   <si>
     <t xml:space="preserve">2 of 2 (100%)</t>

</xml_diff>